<commit_message>
Fix: --quick must not change any exported table
The benchmark table was built with the computed CPA domain scores in a full
run but with the stated 0-3 benchmark values under --quick, so the exported
15_benchmark_0_100.csv depended on which mode had been run last. The flag is
meant to skip figure *rendering* only.

Build the table identically in both modes and regenerate the committed
outputs. Verified: --quick and the full run now produce byte-identical tables,
and both match a clean clone regenerated from scratch.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018DW5967VCybpN1KSSVtrRu
</commit_message>
<xml_diff>
--- a/outputs/tables/posrri_results.xlsx
+++ b/outputs/tables/posrri_results.xlsx
@@ -8170,7 +8170,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>73.33333333333334</v>
+        <v>69.93405530452418</v>
       </c>
       <c r="C2" t="n">
         <v>88.33333333333333</v>
@@ -8189,7 +8189,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>80</v>
+        <v>88.15630755118589</v>
       </c>
       <c r="C3" t="n">
         <v>81.00000000000001</v>
@@ -8208,7 +8208,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>66.66666666666667</v>
+        <v>67.43952714026133</v>
       </c>
       <c r="C4" t="n">
         <v>88</v>
@@ -8227,7 +8227,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>40</v>
+        <v>41.57455978868064</v>
       </c>
       <c r="C5" t="n">
         <v>97</v>
@@ -8246,7 +8246,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>13.33333333333333</v>
+        <v>12.43936410087769</v>
       </c>
       <c r="C6" t="n">
         <v>91</v>
@@ -8265,7 +8265,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>33.33333333333334</v>
+        <v>23.34277051867221</v>
       </c>
       <c r="C7" t="n">
         <v>83.66666666666666</v>
@@ -8284,7 +8284,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>26.66666666666667</v>
+        <v>35.5027021107075</v>
       </c>
       <c r="C8" t="n">
         <v>88.33333333333333</v>
@@ -8303,7 +8303,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>33.33333333333334</v>
+        <v>32.30657908308432</v>
       </c>
       <c r="C9" t="n">
         <v>96.66666666666667</v>
@@ -8322,7 +8322,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>40</v>
+        <v>41.62158004932841</v>
       </c>
       <c r="C10" t="n">
         <v>83.33333333333333</v>
@@ -8341,7 +8341,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>46.66666666666666</v>
+        <v>44.39432783807527</v>
       </c>
       <c r="C11" t="n">
         <v>89.33333333333333</v>

</xml_diff>